<commit_message>
feat(auth): add reset and verify employee functionality with new forms and API endpoints
</commit_message>
<xml_diff>
--- a/employee-import-test.xlsx
+++ b/employee-import-test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13620" windowHeight="5535"/>
+    <workbookView windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>first_name</t>
   </si>
@@ -62,13 +62,13 @@
     <t>Yusuf</t>
   </si>
   <si>
-    <t>amina.yusuf@culturesync.com</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>Customer Support Officer</t>
+    <t>skillmatrix77@gmail.com</t>
+  </si>
+  <si>
+    <t>IT &amp; Infrastructure</t>
+  </si>
+  <si>
+    <t>Software Engineer</t>
   </si>
   <si>
     <t>+2348010000101</t>
@@ -81,66 +81,6 @@
   </si>
   <si>
     <t>2025-03-03</t>
-  </si>
-  <si>
-    <t>David</t>
-  </si>
-  <si>
-    <t>Okafor</t>
-  </si>
-  <si>
-    <t>david.okafor@culturesync.com</t>
-  </si>
-  <si>
-    <t>+2348010000102</t>
-  </si>
-  <si>
-    <t>EMP106</t>
-  </si>
-  <si>
-    <t>2025-03-10</t>
-  </si>
-  <si>
-    <t>Fatima</t>
-  </si>
-  <si>
-    <t>Bello</t>
-  </si>
-  <si>
-    <t>fatima.bello@culturesync.com</t>
-  </si>
-  <si>
-    <t>Executive</t>
-  </si>
-  <si>
-    <t>Sales Executive</t>
-  </si>
-  <si>
-    <t>+2348010000103</t>
-  </si>
-  <si>
-    <t>EMP107</t>
-  </si>
-  <si>
-    <t>2025-03-17</t>
-  </si>
-  <si>
-    <t>Kwame</t>
-  </si>
-  <si>
-    <t>Mensah</t>
-  </si>
-  <si>
-    <t>kwame.mensah@culturesync.com</t>
-  </si>
-  <si>
-    <t>+2348010000104</t>
-  </si>
-  <si>
-    <t>EMP108</t>
-  </si>
-  <si>
-    <t>2025-03-24</t>
   </si>
 </sst>
 </file>
@@ -1368,98 +1308,26 @@
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
+      <c r="B3"/>
+      <c r="C3" s="3"/>
+      <c r="D3"/>
+      <c r="E3"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
+      <c r="B4"/>
+      <c r="C4" s="3"/>
+      <c r="D4"/>
+      <c r="E4"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
-        <v>37</v>
-      </c>
+      <c r="B5"/>
+      <c r="C5" s="3"/>
+      <c r="D5"/>
+      <c r="E5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="amina.yusuf@culturesync.com" tooltip="mailto:amina.yusuf@culturesync.com"/>
-    <hyperlink ref="C3" r:id="rId2" display="david.okafor@culturesync.com" tooltip="mailto:david.okafor@culturesync.com"/>
-    <hyperlink ref="C4" r:id="rId3" display="fatima.bello@culturesync.com"/>
-    <hyperlink ref="C5" r:id="rId4" display="kwame.mensah@culturesync.com"/>
+    <hyperlink ref="C2" r:id="rId1" display="skillmatrix77@gmail.com" tooltip="mailto:skillmatrix77@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>